<commit_message>
update mapping, heatmap and etc
</commit_message>
<xml_diff>
--- a/mapping/mapping_TB2024_v1.xlsx
+++ b/mapping/mapping_TB2024_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khwang/Library/Mobile Documents/com~apple~CloudDocs/Drive/scratch/TB2024/dev_240804_EIC/TB2024/mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CB833B4-CB6B-6343-A148-8CC0E96849A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7F94F2E-E811-744F-B6F2-42D569C9B03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8840" yWindow="6380" windowWidth="29400" windowHeight="18380" xr2:uid="{9904E546-8807-0449-B43D-5949530D5B54}"/>
+    <workbookView xWindow="9180" yWindow="7020" windowWidth="29400" windowHeight="18380" xr2:uid="{9904E546-8807-0449-B43D-5949530D5B54}"/>
   </bookViews>
   <sheets>
     <sheet name="Mapping" sheetId="4" r:id="rId1"/>
@@ -554,7 +554,7 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -571,7 +571,7 @@
         <v>1</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -588,7 +588,7 @@
         <v>1</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -605,7 +605,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -619,10 +619,10 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -639,7 +639,7 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -656,7 +656,7 @@
         <v>2</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -673,7 +673,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -687,10 +687,10 @@
         <v>14</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -704,10 +704,10 @@
         <v>16</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -724,7 +724,7 @@
         <v>3</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -741,7 +741,7 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -755,10 +755,10 @@
         <v>18</v>
       </c>
       <c r="D14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -772,10 +772,10 @@
         <v>19</v>
       </c>
       <c r="D15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -789,10 +789,10 @@
         <v>20</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -805,6 +805,12 @@
       <c r="C17" t="s">
         <v>21</v>
       </c>
+      <c r="D17">
+        <v>4</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18">
@@ -820,7 +826,7 @@
         <v>1</v>
       </c>
       <c r="E18">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -837,7 +843,7 @@
         <v>1</v>
       </c>
       <c r="E19">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -854,7 +860,7 @@
         <v>1</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -871,7 +877,7 @@
         <v>1</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -885,10 +891,10 @@
         <v>26</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -905,7 +911,7 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -922,7 +928,7 @@
         <v>2</v>
       </c>
       <c r="E24">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -939,7 +945,7 @@
         <v>2</v>
       </c>
       <c r="E25">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -953,10 +959,10 @@
         <v>30</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -970,10 +976,10 @@
         <v>31</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -990,7 +996,7 @@
         <v>3</v>
       </c>
       <c r="E28">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1007,7 +1013,7 @@
         <v>3</v>
       </c>
       <c r="E29">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1021,10 +1027,10 @@
         <v>34</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1038,10 +1044,10 @@
         <v>35</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1055,13 +1061,13 @@
         <v>36</v>
       </c>
       <c r="D32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
       <c r="A33">
         <v>1</v>
       </c>
@@ -1071,8 +1077,14 @@
       <c r="C33" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="34" spans="1:3">
+      <c r="D33">
+        <v>4</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
       <c r="A34">
         <v>2</v>
       </c>
@@ -1082,8 +1094,14 @@
       <c r="C34" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="D34">
+        <v>-1</v>
+      </c>
+      <c r="E34">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
       <c r="A35">
         <v>2</v>
       </c>
@@ -1093,8 +1111,14 @@
       <c r="C35" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="36" spans="1:3">
+      <c r="D35">
+        <v>-1</v>
+      </c>
+      <c r="E35">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
       <c r="A36">
         <v>2</v>
       </c>
@@ -1105,7 +1129,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:5">
       <c r="A37">
         <v>2</v>
       </c>
@@ -1116,7 +1140,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:5">
       <c r="A38">
         <v>2</v>
       </c>
@@ -1127,7 +1151,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:5">
       <c r="A39">
         <v>2</v>
       </c>
@@ -1138,7 +1162,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:5">
       <c r="A40">
         <v>2</v>
       </c>
@@ -1149,7 +1173,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:5">
       <c r="A41">
         <v>2</v>
       </c>
@@ -1160,7 +1184,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:5">
       <c r="A42">
         <v>2</v>
       </c>
@@ -1171,7 +1195,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:5">
       <c r="A43">
         <v>2</v>
       </c>
@@ -1182,7 +1206,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:5">
       <c r="A44">
         <v>2</v>
       </c>
@@ -1193,7 +1217,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:5">
       <c r="A45">
         <v>2</v>
       </c>
@@ -1204,7 +1228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:5">
       <c r="A46">
         <v>2</v>
       </c>
@@ -1215,7 +1239,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:5">
       <c r="A47">
         <v>2</v>
       </c>
@@ -1226,7 +1250,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:5">
       <c r="A48">
         <v>2</v>
       </c>
@@ -5066,5 +5090,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>